<commit_message>
Complete F-01 release artifact inventory
</commit_message>
<xml_diff>
--- a/outputs/contract_work_plan_20260630/智慧冰场系统集成工作计划表-细化版.xlsx
+++ b/outputs/contract_work_plan_20260630/智慧冰场系统集成工作计划表-细化版.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能实现" sheetId="1" r:id="Rf1677ab4bcb840a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件界面" sheetId="2" r:id="R966d87e5aac642ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能实现" sheetId="1" r:id="R89ece24ed5884426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="软件界面" sheetId="2" r:id="R95517057010f4242"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -703,7 +703,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -714,7 +714,7 @@
         <x:color rgb="FF854D0E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF9C3"/>
         </x:patternFill>
       </x:fill>
@@ -725,7 +725,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -736,7 +736,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -747,7 +747,7 @@
         <x:color rgb="FF3F6212"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECFCCB"/>
         </x:patternFill>
       </x:fill>
@@ -758,7 +758,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -769,7 +769,7 @@
         <x:color rgb="FF9A3412"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFED7AA"/>
         </x:patternFill>
       </x:fill>
@@ -780,7 +780,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFECACA"/>
         </x:patternFill>
       </x:fill>
@@ -791,7 +791,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -802,7 +802,7 @@
         <x:color rgb="FF854D0E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF9C3"/>
         </x:patternFill>
       </x:fill>
@@ -813,7 +813,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -824,7 +824,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -835,7 +835,7 @@
         <x:color rgb="FF3F6212"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECFCCB"/>
         </x:patternFill>
       </x:fill>
@@ -846,7 +846,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -857,7 +857,7 @@
         <x:color rgb="FF9A3412"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFED7AA"/>
         </x:patternFill>
       </x:fill>
@@ -868,7 +868,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFECACA"/>
         </x:patternFill>
       </x:fill>
@@ -966,9 +966,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1280,13 +1280,13 @@
         <x:v>完整软件系统、部署成果，具备验收条件</x:v>
       </x:c>
       <x:c r="E6" s="44" t="str">
-        <x:v>已有 qmake Release 构建和 post-link 复制规则</x:v>
+        <x:v>已有 qmake Release 构建、post-link 复制规则和 x64/Release 实物目录</x:v>
       </x:c>
       <x:c r="F6" s="44" t="str">
-        <x:v>缺少可交付目录清单和必要/可选文件边界</x:v>
+        <x:v>已补齐可交付目录清单和必要/可选文件边界</x:v>
       </x:c>
       <x:c r="G6" s="44" t="str">
-        <x:v>梳理 exe、Qt 插件、FFmpeg、TensorRT/CUDA DLL、models、配置文件；形成发布目录规范</x:v>
+        <x:v>已梳理 exe、Qt 插件、FFmpeg、TensorRT/CUDA DLL、models、VC Runtime、调试符号/中间目录边界，并写入部署 Runbook</x:v>
       </x:c>
       <x:c r="H6" s="62" t="str">
         <x:v>P0</x:v>
@@ -1295,19 +1295,19 @@
         <x:v>中偏易</x:v>
       </x:c>
       <x:c r="J6" s="44" t="str">
-        <x:v>确认目标交付目录</x:v>
+        <x:v>x64/Release 已存在；目标机目录与 GPU/驱动仍需现场确认</x:v>
       </x:c>
       <x:c r="K6" s="44" t="str">
         <x:v>第1阶段：交付底座</x:v>
       </x:c>
       <x:c r="L6" s="44" t="str">
-        <x:v>交付目录可复制到目标机并启动</x:v>
+        <x:v>按部署 Runbook 复制 x64/Release 到目标机后可启动，并能定位缺失依赖</x:v>
       </x:c>
       <x:c r="M6" s="44" t="str">
-        <x:v>发布包清单</x:v>
+        <x:v>docs/ai-kb/runbooks/deployment.md#Release 发布目录清单</x:v>
       </x:c>
       <x:c r="N6" s="53" t="str">
-        <x:v>不涉及算法</x:v>
+        <x:v>不涉及算法；TensorRT engine 不作为默认跨机交付物</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="56" hidden="0" customHeight="1">
@@ -3001,7 +3001,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0f7a27b5e884d18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c606bd3b9e646cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4585,7 +4585,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb62ec0e83baa4584"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4405a4a8416b4d03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>